<commit_message>
Add specs for drawings 7-12 (Chevrolet Niva, Granta Universal, Largus, Legend, Niva Travel Luxe)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R9zuNWHVAw4QsHcaJhMbSm
</commit_message>
<xml_diff>
--- a/specs/Wiring_3/Wiring_3_spec.xlsx
+++ b/specs/Wiring_3/Wiring_3_spec.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Разъёмы'!$A$1:$M$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Распиновка'!$A$1:$N$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'BOM'!$A$1:$J$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Замечания'!$A$1:$D$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Замечания'!$A$1:$D$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Каталог'!$A$1:$H$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6140,7 +6140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6422,7 +6422,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Гнездо FASTON 41450-1 рассчитано на 2.08–5.26 мм², а провод на листах 2-2…2-4, 3-2…3-4, 6-2 — 1 мм². Обжим будет ненадёжным.</t>
+          <t>Гнездо FASTON 41450-1 рассчитано на 2.08–5.26 мм², а провод на листах 2-2…2-4, 3-2…3-4, 6-2, 10-2…10-4 — 1 мм². Обжим будет ненадёжным.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -6511,8 +6511,28 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Контакты не указаны в BOM</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Для части разъёмов (Yazaki, VAG, Molex NSCC, колодки ВАЗ) контакты в BOM не указаны или указаны без номера.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Подобрать по каталогу производителя корпуса под 0.5–1.0 мм².</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D21"/>
+  <autoFilter ref="A1:D22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>